<commit_message>
feat: add pc list page
</commit_message>
<xml_diff>
--- a/テーブル定義・ER・リレーション図.xlsx
+++ b/テーブル定義・ER・リレーション図.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\大熊 翔\Documents\develop\AssetM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\大熊 翔\Documents\develop\it-asset-manager\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2240354C-F210-424A-8A8B-C22E3CE629B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D15B3763-1378-4312-A186-407DDB4C74FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="改版履歴" sheetId="4" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="109">
   <si>
     <t>テーブル物理名</t>
     <rPh sb="4" eb="6">
@@ -516,6 +516,17 @@
     <rPh sb="0" eb="3">
       <t>リヨウシャ</t>
     </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>貸与物</t>
+    <rPh sb="0" eb="3">
+      <t>タイヨブツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>loaned_items</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -3988,7 +3999,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55727955-9B51-47B2-9611-33FF28EF6908}">
-  <dimension ref="B1:U18"/>
+  <dimension ref="B1:U20"/>
   <sheetFormatPr defaultColWidth="3.25" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="3.25" style="1"/>
@@ -4328,60 +4339,100 @@
       <c r="M15" s="12"/>
     </row>
     <row r="16" spans="2:21" ht="22.15" customHeight="1">
-      <c r="B16" s="22">
+      <c r="B16" s="74">
         <v>8</v>
       </c>
       <c r="C16" s="24" t="s">
-        <v>41</v>
+        <v>107</v>
       </c>
       <c r="D16" s="24" t="s">
-        <v>45</v>
-      </c>
-      <c r="E16" s="24" t="s">
-        <v>67</v>
-      </c>
+        <v>108</v>
+      </c>
+      <c r="E16" s="24"/>
       <c r="F16" s="11"/>
       <c r="G16" s="11"/>
       <c r="H16" s="11"/>
       <c r="I16" s="11"/>
-      <c r="J16" s="11" t="s">
+      <c r="J16" s="11"/>
+      <c r="K16" s="11"/>
+      <c r="L16" s="11"/>
+      <c r="M16" s="12"/>
+    </row>
+    <row r="17" spans="2:13" ht="22.15" customHeight="1">
+      <c r="B17" s="22">
+        <v>9</v>
+      </c>
+      <c r="C17" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="24" t="s">
+        <v>83</v>
+      </c>
+      <c r="E17" s="24"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="11"/>
+      <c r="I17" s="11"/>
+      <c r="J17" s="11"/>
+      <c r="K17" s="11"/>
+      <c r="L17" s="11"/>
+      <c r="M17" s="12"/>
+    </row>
+    <row r="18" spans="2:13" ht="22.15" customHeight="1">
+      <c r="B18" s="74">
+        <v>10</v>
+      </c>
+      <c r="C18" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="D18" s="24" t="s">
+        <v>45</v>
+      </c>
+      <c r="E18" s="24" t="s">
+        <v>67</v>
+      </c>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="11"/>
+      <c r="J18" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="K16" s="11"/>
-      <c r="L16" s="11" t="s">
+      <c r="K18" s="11"/>
+      <c r="L18" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="M16" s="12"/>
-    </row>
-    <row r="17" spans="2:13" ht="22.15" customHeight="1" thickBot="1">
-      <c r="B17" s="23">
-        <v>9</v>
-      </c>
-      <c r="C17" s="25" t="s">
+      <c r="M18" s="12"/>
+    </row>
+    <row r="19" spans="2:13" ht="22.15" customHeight="1" thickBot="1">
+      <c r="B19" s="22">
+        <v>11</v>
+      </c>
+      <c r="C19" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="D17" s="25" t="s">
+      <c r="D19" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="E17" s="25" t="s">
+      <c r="E19" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="F17" s="13"/>
-      <c r="G17" s="13"/>
-      <c r="H17" s="13"/>
-      <c r="I17" s="13"/>
-      <c r="J17" s="13" t="s">
+      <c r="F19" s="13"/>
+      <c r="G19" s="13"/>
+      <c r="H19" s="13"/>
+      <c r="I19" s="13"/>
+      <c r="J19" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="K17" s="13"/>
-      <c r="L17" s="13" t="s">
+      <c r="K19" s="13"/>
+      <c r="L19" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="M17" s="14"/>
-    </row>
-    <row r="18" spans="2:13">
-      <c r="I18" s="3"/>
-      <c r="K18" s="3"/>
+      <c r="M19" s="14"/>
+    </row>
+    <row r="20" spans="2:13">
+      <c r="I20" s="3"/>
+      <c r="K20" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>

</xml_diff>